<commit_message>
Optimize catalogue media, queries, and workbook imports
</commit_message>
<xml_diff>
--- a/client/public/Orange_Catalogue_Direct_Upload_Template.xlsx
+++ b/client/public/Orange_Catalogue_Direct_Upload_Template.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +73,32 @@
       <color rgb="00FFFFFF"/>
       <sz val="17"/>
     </font>
+    <font>
+      <name val="Aptos Display"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="008A623E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="003B3028"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="001F3E65"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -111,8 +135,18 @@
         <fgColor rgb="00EAF3F8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008A623E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -134,11 +168,55 @@
         <color rgb="00E0D6CF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0D6CF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0D6CF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0D6CF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0D6CF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0D6CF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0D6CF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0D6CF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0D6CF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -179,6 +257,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -588,127 +684,127 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="86" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ORANGE CATALOGUE  |  DIRECT EXCEL UPLOAD</t>
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Orange Catalogue — Direct Names + Photos Workbook</t>
         </is>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>This workbook lets staff add customer-facing item names and insert the actual product photos into Excel. Upload the completed workbook in Admin → POS imports → Direct catalogue workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>HOW TO COMPLETE THIS WORKBOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>First import the latest POS inventory file into the website. This ensures every cleaned code and POS Attribute colour exists.</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Open “Catalogue Upload”. Add one row for each product name or photo. Use the exact Cleaned Code shown in the website.</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>For a product name, enter the Cleaned Code and Website Name. The name is saved once for the whole item, even if it has several colours.</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>For a photo, enter the Cleaned Code and exact POS Attribute Colour, then click the “Embedded Photo” cell and use Excel Insert → Pictures to place the real image in that cell area.</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Use one photo per row. To add a second photo for the same colour, create another row and repeat the same Cleaned Code and POS Attribute Colour.</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Do not rename POS colours, paste a website link, or add photos outside the “Embedded Photo” column. Save as .xlsx, then upload it through the Direct catalogue workbook area.</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-    </row>
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>How to use this workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>1. Import inventory first</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Upload the current POS inventory file in the Orange admin area before using this workbook. The website matches each row to that imported POS item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>2. Keep the exact Cleaned Code</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Copy the existing Cleaned Code and POS Attribute Colour exactly. Do not change the header names or move the Embedded Photo column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>3. Add the website name</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Enter the customer-facing Website Name once for each product model. Repeated colour rows may use the same name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>4. Insert the real photo</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Place the original JPG, PNG, or WebP directly inside the blue Embedded Photo column. Do not paste screenshots or compressed Messenger copies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>5. Preserve image quality</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Turn off Excel picture compression if available. The picture’s displayed cell size does not reduce the uploaded source quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>6. Use manageable batches</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>For smooth imports, use a category or collection per workbook: about 50–100 photos or less than 20 MB total. Split larger batches into separate workbooks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>7. Reuse and replacement</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>The same photo is recognised and reused without another upload. In the admin preview, tick Replace older photos only when the workbook contains the complete new set for those colours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>8. Preview before upload</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Upload the workbook in Admin → POS imports → Direct catalogue workbook. Review all matches and warnings before applying. Failed photos can be retried without re-sending successful photos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
@@ -716,6 +812,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -734,9 +831,6 @@
           <t>The file is saved as .xlsx.</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -749,9 +843,6 @@
           <t>The latest POS inventory was imported first.</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -764,9 +855,6 @@
           <t>Every row has a Cleaned Code.</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
     </row>
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -779,9 +867,6 @@
           <t>Every photo row has the exact POS Attribute Colour.</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
@@ -794,28 +879,28 @@
           <t>Every photo is inserted in the blue Embedded Photo column.</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-    </row>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="A3:E3"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -843,6 +928,11 @@
           <t>CATALOGUE UPLOAD  |  NAMES + EMBEDDED PHOTOS</t>
         </is>
       </c>
+      <c r="E1" s="23" t="inlineStr">
+        <is>
+          <t>Embedded Photo</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
@@ -1601,10 +1691,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A6:E106"/>
-  <mergeCells count="2">
-    <mergeCell ref="A3:E4"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>